<commit_message>
Updated some assertions of the spi slave
</commit_message>
<xml_diff>
--- a/verification plan/verification plan.xlsx
+++ b/verification plan/verification plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Shared Folders\Uni\courses\Digital circuit\digital github codes\Done\spi\Verification-of-SPI-Slave-with-Single-Port-RAM\verification plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F324BD-735A-4AA9-A044-B39EFB798289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B79B1A-5A46-47B2-9A89-4FF0635B1F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30" yWindow="30" windowWidth="28770" windowHeight="15450" xr2:uid="{BE33C207-AC50-49BB-BEDD-1F59C983F64D}"/>
   </bookViews>
@@ -1242,7 +1242,7 @@
         <v>100</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="K4" s="7"/>
     </row>
@@ -1401,7 +1401,7 @@
         <v>100</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="K10" s="7"/>
     </row>

</xml_diff>

<commit_message>
Added assertion sections 4 and 5, as outlined in the verification plan
</commit_message>
<xml_diff>
--- a/verification plan/verification plan.xlsx
+++ b/verification plan/verification plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Shared Folders\Uni\courses\Digital circuit\digital github codes\Done\spi\Verification-of-SPI-Slave-with-Single-Port-RAM\verification plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B79B1A-5A46-47B2-9A89-4FF0635B1F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E6DC00-F6E6-465F-853D-9A5D15C2ED43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="30" windowWidth="28770" windowHeight="15450" xr2:uid="{BE33C207-AC50-49BB-BEDD-1F59C983F64D}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{BE33C207-AC50-49BB-BEDD-1F59C983F64D}"/>
   </bookViews>
   <sheets>
     <sheet name="Verification Plan" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="154">
   <si>
     <t>#</t>
   </si>
@@ -545,6 +545,9 @@
   </si>
   <si>
     <t>Concurrent assertion to check for the writen data on the internal array mem of the RAM</t>
+  </si>
+  <si>
+    <t>Assertion: assert_idle</t>
   </si>
 </sst>
 </file>
@@ -1370,7 +1373,7 @@
         <v>100</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="K9" s="7"/>
     </row>
@@ -1432,7 +1435,7 @@
         <v>100</v>
       </c>
       <c r="J11" s="12" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="K11" s="7"/>
     </row>
@@ -1463,7 +1466,7 @@
         <v>100</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="K12" s="7"/>
     </row>
@@ -1556,7 +1559,7 @@
         <v>100</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="K15" s="7"/>
     </row>
@@ -1618,7 +1621,7 @@
         <v>100</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="K17" s="7"/>
     </row>
@@ -1680,7 +1683,7 @@
         <v>100</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="K19" s="7"/>
     </row>
@@ -1744,7 +1747,7 @@
         <v>70</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>30</v>
+        <v>153</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>73</v>

</xml_diff>